<commit_message>
output 4 and 5
</commit_message>
<xml_diff>
--- a/output_5a.xlsx
+++ b/output_5a.xlsx
@@ -1102,7 +1102,7 @@
         <v>13</v>
       </c>
       <c r="B14" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="C14" t="n">
         <v>-0</v>
@@ -1111,7 +1111,7 @@
         <v>-0</v>
       </c>
       <c r="E14" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="F14" t="n">
         <v>-0</v>
@@ -1122,7 +1122,7 @@
         <v>14</v>
       </c>
       <c r="B15" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="C15" t="n">
         <v>-0</v>
@@ -1131,7 +1131,7 @@
         <v>-0</v>
       </c>
       <c r="E15" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="F15" t="n">
         <v>-0</v>
@@ -1165,16 +1165,16 @@
         <v>0</v>
       </c>
       <c r="C17" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="D17" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="E17" t="n">
         <v>0</v>
       </c>
       <c r="F17" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
     </row>
     <row r="18">

</xml_diff>